<commit_message>
chore(output): refresh the committed analysis baseline
The tracked outputs were produced by an older fork build: risks.json had no
risk_status/risk_explanation fields and no source column, so CI's risk diff
compared fresh results against a stale schema and the committed scorecard
still showed 99% completeness (the llm-summarizer boundary gap). Regenerate
the CI-diffed files (risks.json, risks.xlsx, tags.xlsx, stats.json,
technical-assets.json) and the derived reports (score.md, summary.md,
prioritized-findings.md); score-badge.json and the security-requirements
files came out byte-identical.

The risk set is unchanged (67 findings, score 81/100 grade B) — the
differences are the applied tracking statuses, the completed trust-boundary
coverage (100% now) and the updated schema. Presentation artifacts that
need Graphviz (report.pdf, the adoc export, diagram PNGs) and the
per-methodology directories are left for the CI baseline job, which has
Graphviz installed.
</commit_message>
<xml_diff>
--- a/threagile/output/tags.xlsx
+++ b/threagile/output/tags.xlsx
@@ -316,149 +316,127 @@
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:ap="http://schemas.openxmlformats.org/officeDocument/2006/extended-properties" xmlns:op="http://schemas.openxmlformats.org/officeDocument/2006/custom-properties" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cdr="http://schemas.openxmlformats.org/drawingml/2006/chartDrawing" xmlns:comp="http://schemas.openxmlformats.org/drawingml/2006/compatibility" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:lc="http://schemas.openxmlformats.org/drawingml/2006/lockedCanvas" xmlns:pic="http://schemas.openxmlformats.org/drawingml/2006/picture" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" xmlns:m="http://schemas.openxmlformats.org/officeDocument/2006/math" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:sl="http://schemas.openxmlformats.org/schemaLibrary/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xne="http://schemas.microsoft.com/office/excel/2006/main" xmlns:mso="http://schemas.microsoft.com/office/2006/01/customui" xmlns:ax="http://schemas.microsoft.com/office/2006/activeX" xmlns:cppr="http://schemas.microsoft.com/office/2006/coverPageProps" xmlns:cdip="http://schemas.microsoft.com/office/2006/customDocumentInformationPanel" xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ntns="http://schemas.microsoft.com/office/2006/metadata/customXsn" xmlns:lp="http://schemas.microsoft.com/office/2006/metadata/longProperties" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" xmlns:msink="http://schemas.microsoft.com/ink/2010/main" xmlns:c14="http://schemas.microsoft.com/office/drawing/2007/8/2/chart" xmlns:cdr14="http://schemas.microsoft.com/office/drawing/2010/chartDrawing" xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" xmlns:pic14="http://schemas.microsoft.com/office/drawing/2010/picture" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xdr14="http://schemas.microsoft.com/office/excel/2010/spreadsheetDrawing" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:dsp="http://schemas.microsoft.com/office/drawing/2008/diagram" xmlns:mso14="http://schemas.microsoft.com/office/2009/07/customui" xmlns:dgm14="http://schemas.microsoft.com/office/drawing/2010/diagram" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x12ac="http://schemas.microsoft.com/office/spreadsheetml/2011/1/ac" xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" xmlns:xr4="http://schemas.microsoft.com/office/spreadsheetml/2016/revision4" xmlns:xr5="http://schemas.microsoft.com/office/spreadsheetml/2016/revision5" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr7="http://schemas.microsoft.com/office/spreadsheetml/2016/revision7" xmlns:xr8="http://schemas.microsoft.com/office/spreadsheetml/2016/revision8" xmlns:xr9="http://schemas.microsoft.com/office/spreadsheetml/2016/revision9" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr11="http://schemas.microsoft.com/office/spreadsheetml/2016/revision11" xmlns:xr12="http://schemas.microsoft.com/office/spreadsheetml/2016/revision12" xmlns:xr13="http://schemas.microsoft.com/office/spreadsheetml/2016/revision13" xmlns:xr14="http://schemas.microsoft.com/office/spreadsheetml/2016/revision14" xmlns:xr15="http://schemas.microsoft.com/office/spreadsheetml/2016/revision15" xmlns:x16="http://schemas.microsoft.com/office/spreadsheetml/2014/11/main" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:mo="http://schemas.microsoft.com/office/mac/office/2008/main" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:o="urn:schemas-microsoft-com:office:office" xmlns:v="urn:schemas-microsoft-com:vml" mc:Ignorable="c14 cdr14 a14 pic14 x14 xdr14 x14ac dsp mso14 dgm14 x15 x12ac x15ac xr xr2 xr3 xr4 xr5 xr6 xr7 xr8 xr9 xr10 xr11 xr12 xr13 xr14 xr15 x15 x16 x16r2 mo mx mv o v" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <fonts count="23">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
+      <color theme="1"/>
+      <sz val="11"/>
     </font>
     <font>
+      <family val="2"/>
       <b val="1"/>
+      <color rgb="FFFF2600"/>
       <sz val="12"/>
-      <color rgb="FFFF2600"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FFFF2600"/>
       <sz val="12"/>
-      <color rgb="FFFF2600"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
       <b val="1"/>
+      <color rgb="FFA0281E"/>
       <sz val="12"/>
-      <color rgb="FFA0281E"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FFA0281E"/>
       <sz val="12"/>
-      <color rgb="FFA0281E"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
       <b val="1"/>
+      <color rgb="FFFF8E00"/>
       <sz val="12"/>
-      <color rgb="FFFF8E00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FFFF8E00"/>
       <sz val="12"/>
-      <color rgb="FFFF8E00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
       <b val="1"/>
+      <color rgb="FFC87832"/>
       <sz val="12"/>
-      <color rgb="FFC87832"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FFC87832"/>
       <sz val="12"/>
-      <color rgb="FFC87832"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
       <b val="1"/>
+      <color rgb="FF23465F"/>
       <sz val="12"/>
-      <color rgb="FF23465F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FF23465F"/>
       <sz val="12"/>
-      <color rgb="FF23465F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FF008F00"/>
       <sz val="12"/>
-      <color rgb="FF008F00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FF0000FF"/>
       <sz val="12"/>
-      <color rgb="FF0000FF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FFFF40FF"/>
       <sz val="12"/>
-      <color rgb="FFFF40FF"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FFFF9300"/>
       <sz val="12"/>
-      <color rgb="FFFF9300"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FF666666"/>
       <sz val="12"/>
-      <color rgb="FF666666"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="10"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FF7F7F7F"/>
       <sz val="10"/>
-      <color rgb="FF7F7F7F"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
       <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="12"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FF008F00"/>
       <sz val="10"/>
-      <color rgb="FF008F00"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
       <b val="1"/>
+      <color rgb="FF000000"/>
       <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
     <font>
+      <family val="2"/>
+      <color rgb="FF000000"/>
       <sz val="14"/>
-      <color rgb="FF000000"/>
-      <name val="Calibri"/>
-      <family val="2"/>
     </font>
   </fonts>
   <fills count="3">

</xml_diff>